<commit_message>
Add player Elo system, Elo-only model, and retrain on Masters Santiago data
- Add player_elo.py: ranking Elo system with role-normalised composite scores,
  own_factor² dampening, K=64, change range 15-30 (tuned via hyperparam search)
- Add feature_engineering_elo.py: minimal 3-feature model (ranking_elo_sum_diff,
  ranking_elo_trend_diff, fk_fd_diff_overall_5_diff)
- Add elo_hyperparam_search.py: grid search over K/min/max Elo params
- Update feature_engineering_v3.py: add Elo features and match_id to full pipeline
- Update train_model.py: add --input flag, add match_id to non-feature cols
- Update predict.py: integrate Elo features, display per-player Elo and FK/FD diff
- Retrain model on updated data including Masters Santiago 2026 (58.8% accuracy)

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Model Accuracy Tracking.xlsx
+++ b/Model Accuracy Tracking.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jdl11\Desktop\VPM\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45451433-8C6A-4A8D-949D-63F0A87E0AE2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6CC4560B-A206-4CB6-B534-8D330B4F2E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{340DB975-8699-4957-AF02-B724CDF6AF4C}"/>
   </bookViews>
@@ -59,7 +59,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="192" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="252" uniqueCount="54">
   <si>
     <t>Team A</t>
   </si>
@@ -616,7 +616,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B7028733-08D0-4678-B1C6-873990459FB9}">
-  <dimension ref="A1:N36"/>
+  <dimension ref="A1:N55"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="2" width="11.54296875" bestFit="1" customWidth="1"/>
@@ -1909,22 +1909,22 @@
         <v>38</v>
       </c>
       <c r="F29">
-        <f t="shared" ref="F29:F36" si="12">IF(D29=E29,1,0)</f>
+        <f t="shared" ref="F29:F55" si="12">IF(D29=E29,1,0)</f>
         <v>1</v>
       </c>
       <c r="G29" s="4">
         <v>0.60299999999999998</v>
       </c>
       <c r="H29" s="1">
-        <f t="shared" ref="H29:H36" si="13">1-G29</f>
+        <f t="shared" ref="H29:H55" si="13">1-G29</f>
         <v>0.39700000000000002</v>
       </c>
       <c r="I29" s="1">
-        <f t="shared" ref="I29:I36" si="14">IF(K29&lt;0,(-K29)/((-K29)+100),100/(K29+100))</f>
+        <f t="shared" ref="I29:I55" si="14">IF(K29&lt;0,(-K29)/((-K29)+100),100/(K29+100))</f>
         <v>1</v>
       </c>
       <c r="J29" s="1">
-        <f t="shared" ref="J29:J36" si="15">IF(L29&lt;0,(-L29)/((-L29)+100),100/(L29+100))</f>
+        <f t="shared" ref="J29:J55" si="15">IF(L29&lt;0,(-L29)/((-L29)+100),100/(L29+100))</f>
         <v>1</v>
       </c>
       <c r="K29" s="6"/>
@@ -1935,14 +1935,31 @@
       </c>
     </row>
     <row r="30" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A30" t="s">
+        <v>51</v>
+      </c>
+      <c r="B30" t="s">
+        <v>9</v>
+      </c>
+      <c r="C30" t="s">
+        <v>31</v>
+      </c>
+      <c r="D30" t="s">
+        <v>51</v>
+      </c>
+      <c r="E30" t="s">
+        <v>51</v>
+      </c>
       <c r="F30">
         <f t="shared" si="12"/>
         <v>1</v>
       </c>
-      <c r="G30" s="4"/>
+      <c r="G30" s="4">
+        <v>0.57099999999999995</v>
+      </c>
       <c r="H30" s="1">
         <f t="shared" si="13"/>
-        <v>1</v>
+        <v>0.42900000000000005</v>
       </c>
       <c r="I30" s="1">
         <f t="shared" si="14"/>
@@ -1960,14 +1977,31 @@
       </c>
     </row>
     <row r="31" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A31" t="s">
+        <v>51</v>
+      </c>
+      <c r="B31" t="s">
+        <v>9</v>
+      </c>
+      <c r="C31" t="s">
+        <v>36</v>
+      </c>
+      <c r="D31" t="s">
+        <v>9</v>
+      </c>
+      <c r="E31" t="s">
+        <v>51</v>
+      </c>
       <c r="F31">
         <f t="shared" si="12"/>
-        <v>1</v>
-      </c>
-      <c r="G31" s="4"/>
+        <v>0</v>
+      </c>
+      <c r="G31" s="4">
+        <v>0.51700000000000002</v>
+      </c>
       <c r="H31" s="1">
         <f t="shared" si="13"/>
-        <v>1</v>
+        <v>0.48299999999999998</v>
       </c>
       <c r="I31" s="1">
         <f t="shared" si="14"/>
@@ -1985,14 +2019,31 @@
       </c>
     </row>
     <row r="32" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A32" t="s">
+        <v>8</v>
+      </c>
+      <c r="B32" t="s">
+        <v>38</v>
+      </c>
+      <c r="C32" t="s">
+        <v>21</v>
+      </c>
+      <c r="D32" t="s">
+        <v>38</v>
+      </c>
+      <c r="E32" t="s">
+        <v>38</v>
+      </c>
       <c r="F32">
         <f t="shared" si="12"/>
         <v>1</v>
       </c>
-      <c r="G32" s="4"/>
+      <c r="G32" s="4">
+        <v>0.439</v>
+      </c>
       <c r="H32" s="1">
         <f t="shared" si="13"/>
-        <v>1</v>
+        <v>0.56099999999999994</v>
       </c>
       <c r="I32" s="1">
         <f t="shared" si="14"/>
@@ -2009,15 +2060,32 @@
         <v>No</v>
       </c>
     </row>
-    <row r="33" spans="6:13" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A33" t="s">
+        <v>8</v>
+      </c>
+      <c r="B33" t="s">
+        <v>38</v>
+      </c>
+      <c r="C33" t="s">
+        <v>34</v>
+      </c>
+      <c r="D33" t="s">
+        <v>8</v>
+      </c>
+      <c r="E33" t="s">
+        <v>8</v>
+      </c>
       <c r="F33">
         <f t="shared" si="12"/>
         <v>1</v>
       </c>
-      <c r="G33" s="4"/>
+      <c r="G33" s="4">
+        <v>0.56299999999999994</v>
+      </c>
       <c r="H33" s="1">
         <f t="shared" si="13"/>
-        <v>1</v>
+        <v>0.43700000000000006</v>
       </c>
       <c r="I33" s="1">
         <f t="shared" si="14"/>
@@ -2034,15 +2102,32 @@
         <v>No</v>
       </c>
     </row>
-    <row r="34" spans="6:13" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A34" t="s">
+        <v>8</v>
+      </c>
+      <c r="B34" t="s">
+        <v>38</v>
+      </c>
+      <c r="C34" t="s">
+        <v>52</v>
+      </c>
+      <c r="D34" t="s">
+        <v>8</v>
+      </c>
+      <c r="E34" t="s">
+        <v>8</v>
+      </c>
       <c r="F34">
         <f t="shared" si="12"/>
         <v>1</v>
       </c>
-      <c r="G34" s="4"/>
+      <c r="G34" s="4">
+        <v>0.59099999999999997</v>
+      </c>
       <c r="H34" s="1">
         <f t="shared" si="13"/>
-        <v>1</v>
+        <v>0.40900000000000003</v>
       </c>
       <c r="I34" s="1">
         <f t="shared" si="14"/>
@@ -2059,15 +2144,32 @@
         <v>No</v>
       </c>
     </row>
-    <row r="35" spans="6:13" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A35" t="s">
+        <v>9</v>
+      </c>
+      <c r="B35" t="s">
+        <v>8</v>
+      </c>
+      <c r="C35" t="s">
+        <v>20</v>
+      </c>
+      <c r="D35" t="s">
+        <v>9</v>
+      </c>
+      <c r="E35" t="s">
+        <v>9</v>
+      </c>
       <c r="F35">
         <f t="shared" si="12"/>
         <v>1</v>
       </c>
-      <c r="G35" s="4"/>
+      <c r="G35" s="4">
+        <v>0.56200000000000006</v>
+      </c>
       <c r="H35" s="1">
         <f t="shared" si="13"/>
-        <v>1</v>
+        <v>0.43799999999999994</v>
       </c>
       <c r="I35" s="1">
         <f t="shared" si="14"/>
@@ -2084,15 +2186,32 @@
         <v>No</v>
       </c>
     </row>
-    <row r="36" spans="6:13" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A36" t="s">
+        <v>9</v>
+      </c>
+      <c r="B36" t="s">
+        <v>8</v>
+      </c>
+      <c r="C36" t="s">
+        <v>5</v>
+      </c>
+      <c r="D36" t="s">
+        <v>8</v>
+      </c>
+      <c r="E36" t="s">
+        <v>8</v>
+      </c>
       <c r="F36">
         <f t="shared" si="12"/>
         <v>1</v>
       </c>
-      <c r="G36" s="4"/>
+      <c r="G36" s="4">
+        <v>0.42499999999999999</v>
+      </c>
       <c r="H36" s="1">
         <f t="shared" si="13"/>
-        <v>1</v>
+        <v>0.57499999999999996</v>
       </c>
       <c r="I36" s="1">
         <f t="shared" si="14"/>
@@ -2106,6 +2225,566 @@
       <c r="L36" s="6"/>
       <c r="M36" t="str" cm="1">
         <f t="array" ref="M36">_xlfn.IFS(G36&gt;I36,"Team A",H36&gt;J36,"Team B",TRUE,"No")</f>
+        <v>No</v>
+      </c>
+    </row>
+    <row r="37" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A37" t="s">
+        <v>9</v>
+      </c>
+      <c r="B37" t="s">
+        <v>8</v>
+      </c>
+      <c r="C37" t="s">
+        <v>52</v>
+      </c>
+      <c r="D37" t="s">
+        <v>8</v>
+      </c>
+      <c r="E37" t="s">
+        <v>8</v>
+      </c>
+      <c r="F37">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="G37" s="4">
+        <v>0.44700000000000001</v>
+      </c>
+      <c r="H37" s="1">
+        <f t="shared" si="13"/>
+        <v>0.55299999999999994</v>
+      </c>
+      <c r="I37" s="1">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="J37" s="1">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="K37" s="6"/>
+      <c r="L37" s="6"/>
+      <c r="M37" t="str" cm="1">
+        <f t="array" ref="M37">_xlfn.IFS(G37&gt;I37,"Team A",H37&gt;J37,"Team B",TRUE,"No")</f>
+        <v>No</v>
+      </c>
+    </row>
+    <row r="38" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A38" t="s">
+        <v>9</v>
+      </c>
+      <c r="B38" t="s">
+        <v>8</v>
+      </c>
+      <c r="C38" t="s">
+        <v>34</v>
+      </c>
+      <c r="D38" t="s">
+        <v>8</v>
+      </c>
+      <c r="E38" t="s">
+        <v>8</v>
+      </c>
+      <c r="F38">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="G38" s="4">
+        <v>0.40899999999999997</v>
+      </c>
+      <c r="H38" s="1">
+        <f t="shared" si="13"/>
+        <v>0.59099999999999997</v>
+      </c>
+      <c r="I38" s="1">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="J38" s="1">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="K38" s="6"/>
+      <c r="L38" s="6"/>
+      <c r="M38" t="str" cm="1">
+        <f t="array" ref="M38">_xlfn.IFS(G38&gt;I38,"Team A",H38&gt;J38,"Team B",TRUE,"No")</f>
+        <v>No</v>
+      </c>
+    </row>
+    <row r="39" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A39" t="s">
+        <v>51</v>
+      </c>
+      <c r="B39" t="s">
+        <v>8</v>
+      </c>
+      <c r="C39" t="s">
+        <v>52</v>
+      </c>
+      <c r="D39" t="s">
+        <v>8</v>
+      </c>
+      <c r="E39" t="s">
+        <v>51</v>
+      </c>
+      <c r="F39">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="G39" s="4">
+        <v>0.41399999999999998</v>
+      </c>
+      <c r="H39" s="1">
+        <f t="shared" si="13"/>
+        <v>0.58600000000000008</v>
+      </c>
+      <c r="I39" s="1">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="J39" s="1">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="K39" s="6"/>
+      <c r="L39" s="6"/>
+      <c r="M39" t="str" cm="1">
+        <f t="array" ref="M39">_xlfn.IFS(G39&gt;I39,"Team A",H39&gt;J39,"Team B",TRUE,"No")</f>
+        <v>No</v>
+      </c>
+    </row>
+    <row r="40" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A40" t="s">
+        <v>51</v>
+      </c>
+      <c r="B40" t="s">
+        <v>8</v>
+      </c>
+      <c r="C40" t="s">
+        <v>5</v>
+      </c>
+      <c r="D40" t="s">
+        <v>8</v>
+      </c>
+      <c r="E40" t="s">
+        <v>51</v>
+      </c>
+      <c r="F40">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="G40" s="4">
+        <v>0.436</v>
+      </c>
+      <c r="H40" s="1">
+        <f t="shared" si="13"/>
+        <v>0.56400000000000006</v>
+      </c>
+      <c r="I40" s="1">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="J40" s="1">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="K40" s="6"/>
+      <c r="L40" s="6"/>
+      <c r="M40" t="str" cm="1">
+        <f t="array" ref="M40">_xlfn.IFS(G40&gt;I40,"Team A",H40&gt;J40,"Team B",TRUE,"No")</f>
+        <v>No</v>
+      </c>
+    </row>
+    <row r="41" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A41" t="s">
+        <v>51</v>
+      </c>
+      <c r="B41" t="s">
+        <v>8</v>
+      </c>
+      <c r="C41" t="s">
+        <v>36</v>
+      </c>
+      <c r="D41" t="s">
+        <v>8</v>
+      </c>
+      <c r="E41" t="s">
+        <v>51</v>
+      </c>
+      <c r="F41">
+        <f t="shared" si="12"/>
+        <v>0</v>
+      </c>
+      <c r="G41" s="4">
+        <v>0.42299999999999999</v>
+      </c>
+      <c r="H41" s="1">
+        <f t="shared" si="13"/>
+        <v>0.57699999999999996</v>
+      </c>
+      <c r="I41" s="1">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="J41" s="1">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="K41" s="6"/>
+      <c r="L41" s="6"/>
+      <c r="M41" t="str" cm="1">
+        <f t="array" ref="M41">_xlfn.IFS(G41&gt;I41,"Team A",H41&gt;J41,"Team B",TRUE,"No")</f>
+        <v>No</v>
+      </c>
+    </row>
+    <row r="42" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="F42">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="G42" s="4"/>
+      <c r="H42" s="1">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="I42" s="1">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="J42" s="1">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="K42" s="6"/>
+      <c r="L42" s="6"/>
+      <c r="M42" t="str" cm="1">
+        <f t="array" ref="M42">_xlfn.IFS(G42&gt;I42,"Team A",H42&gt;J42,"Team B",TRUE,"No")</f>
+        <v>No</v>
+      </c>
+    </row>
+    <row r="43" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="F43">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="G43" s="4"/>
+      <c r="H43" s="1">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="I43" s="1">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="J43" s="1">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="K43" s="6"/>
+      <c r="L43" s="6"/>
+      <c r="M43" t="str" cm="1">
+        <f t="array" ref="M43">_xlfn.IFS(G43&gt;I43,"Team A",H43&gt;J43,"Team B",TRUE,"No")</f>
+        <v>No</v>
+      </c>
+    </row>
+    <row r="44" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="F44">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="G44" s="4"/>
+      <c r="H44" s="1">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="I44" s="1">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="J44" s="1">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="K44" s="6"/>
+      <c r="L44" s="6"/>
+      <c r="M44" t="str" cm="1">
+        <f t="array" ref="M44">_xlfn.IFS(G44&gt;I44,"Team A",H44&gt;J44,"Team B",TRUE,"No")</f>
+        <v>No</v>
+      </c>
+    </row>
+    <row r="45" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="F45">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="G45" s="4"/>
+      <c r="H45" s="1">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="I45" s="1">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="J45" s="1">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="K45" s="6"/>
+      <c r="L45" s="6"/>
+      <c r="M45" t="str" cm="1">
+        <f t="array" ref="M45">_xlfn.IFS(G45&gt;I45,"Team A",H45&gt;J45,"Team B",TRUE,"No")</f>
+        <v>No</v>
+      </c>
+    </row>
+    <row r="46" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="F46">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="G46" s="4"/>
+      <c r="H46" s="1">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="I46" s="1">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="J46" s="1">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="K46" s="6"/>
+      <c r="L46" s="6"/>
+      <c r="M46" t="str" cm="1">
+        <f t="array" ref="M46">_xlfn.IFS(G46&gt;I46,"Team A",H46&gt;J46,"Team B",TRUE,"No")</f>
+        <v>No</v>
+      </c>
+    </row>
+    <row r="47" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="F47">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="G47" s="4"/>
+      <c r="H47" s="1">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="I47" s="1">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="J47" s="1">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="K47" s="6"/>
+      <c r="L47" s="6"/>
+      <c r="M47" t="str" cm="1">
+        <f t="array" ref="M47">_xlfn.IFS(G47&gt;I47,"Team A",H47&gt;J47,"Team B",TRUE,"No")</f>
+        <v>No</v>
+      </c>
+    </row>
+    <row r="48" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="F48">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="G48" s="4"/>
+      <c r="H48" s="1">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="I48" s="1">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="J48" s="1">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="K48" s="6"/>
+      <c r="L48" s="6"/>
+      <c r="M48" t="str" cm="1">
+        <f t="array" ref="M48">_xlfn.IFS(G48&gt;I48,"Team A",H48&gt;J48,"Team B",TRUE,"No")</f>
+        <v>No</v>
+      </c>
+    </row>
+    <row r="49" spans="6:13" x14ac:dyDescent="0.35">
+      <c r="F49">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="G49" s="4"/>
+      <c r="H49" s="1">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="I49" s="1">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="J49" s="1">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="K49" s="6"/>
+      <c r="L49" s="6"/>
+      <c r="M49" t="str" cm="1">
+        <f t="array" ref="M49">_xlfn.IFS(G49&gt;I49,"Team A",H49&gt;J49,"Team B",TRUE,"No")</f>
+        <v>No</v>
+      </c>
+    </row>
+    <row r="50" spans="6:13" x14ac:dyDescent="0.35">
+      <c r="F50">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="G50" s="4"/>
+      <c r="H50" s="1">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="I50" s="1">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="J50" s="1">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="K50" s="6"/>
+      <c r="L50" s="6"/>
+      <c r="M50" t="str" cm="1">
+        <f t="array" ref="M50">_xlfn.IFS(G50&gt;I50,"Team A",H50&gt;J50,"Team B",TRUE,"No")</f>
+        <v>No</v>
+      </c>
+    </row>
+    <row r="51" spans="6:13" x14ac:dyDescent="0.35">
+      <c r="F51">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="G51" s="4"/>
+      <c r="H51" s="1">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="I51" s="1">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="J51" s="1">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="K51" s="6"/>
+      <c r="L51" s="6"/>
+      <c r="M51" t="str" cm="1">
+        <f t="array" ref="M51">_xlfn.IFS(G51&gt;I51,"Team A",H51&gt;J51,"Team B",TRUE,"No")</f>
+        <v>No</v>
+      </c>
+    </row>
+    <row r="52" spans="6:13" x14ac:dyDescent="0.35">
+      <c r="F52">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="G52" s="4"/>
+      <c r="H52" s="1">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="I52" s="1">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="J52" s="1">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="K52" s="6"/>
+      <c r="L52" s="6"/>
+      <c r="M52" t="str" cm="1">
+        <f t="array" ref="M52">_xlfn.IFS(G52&gt;I52,"Team A",H52&gt;J52,"Team B",TRUE,"No")</f>
+        <v>No</v>
+      </c>
+    </row>
+    <row r="53" spans="6:13" x14ac:dyDescent="0.35">
+      <c r="F53">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="G53" s="4"/>
+      <c r="H53" s="1">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="I53" s="1">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="J53" s="1">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="K53" s="6"/>
+      <c r="L53" s="6"/>
+      <c r="M53" t="str" cm="1">
+        <f t="array" ref="M53">_xlfn.IFS(G53&gt;I53,"Team A",H53&gt;J53,"Team B",TRUE,"No")</f>
+        <v>No</v>
+      </c>
+    </row>
+    <row r="54" spans="6:13" x14ac:dyDescent="0.35">
+      <c r="F54">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="G54" s="4"/>
+      <c r="H54" s="1">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="I54" s="1">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="J54" s="1">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="K54" s="6"/>
+      <c r="L54" s="6"/>
+      <c r="M54" t="str" cm="1">
+        <f t="array" ref="M54">_xlfn.IFS(G54&gt;I54,"Team A",H54&gt;J54,"Team B",TRUE,"No")</f>
+        <v>No</v>
+      </c>
+    </row>
+    <row r="55" spans="6:13" x14ac:dyDescent="0.35">
+      <c r="F55">
+        <f t="shared" si="12"/>
+        <v>1</v>
+      </c>
+      <c r="G55" s="4"/>
+      <c r="H55" s="1">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="I55" s="1">
+        <f t="shared" si="14"/>
+        <v>1</v>
+      </c>
+      <c r="J55" s="1">
+        <f t="shared" si="15"/>
+        <v>1</v>
+      </c>
+      <c r="K55" s="6"/>
+      <c r="L55" s="6"/>
+      <c r="M55" t="str" cm="1">
+        <f t="array" ref="M55">_xlfn.IFS(G55&gt;I55,"Team A",H55&gt;J55,"Team B",TRUE,"No")</f>
         <v>No</v>
       </c>
     </row>

</xml_diff>